<commit_message>
Add live show sponsorship sheet to the model
New Live show sheet builds the weekly show's sponsor revenue bottom up from
Noa's tiers ($10k Presented By, $8k and $6k banners) with floor, base and
ceiling cases and a slot cap per show (Presented By is 1 per show).

By default the show sits inside the existing sponsor lines, so deck totals
are unchanged ($430k, $3.4M, $8.0M, $22.6M) and the Dashboard shows how much
of the sponsorship forecast the show backs. Treatment 2 adds it on top.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/workspace/model.xlsx
+++ b/public/workspace/model.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -10,7 +10,8 @@
   <sheets>
     <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="PnL" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Live show" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="PnL" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="158">
   <si>
     <t xml:space="preserve">BEYOND TOMORROW FINANCIAL MODEL</t>
   </si>
@@ -78,6 +79,18 @@
     <t xml:space="preserve">Any FAIL above means an input no longer ties; check the yellow cells on Assumptions.</t>
   </si>
   <si>
+    <t xml:space="preserve">Live show sponsorship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sponsorship still to be won</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of sponsorship backed by the show</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live show checks all pass</t>
+  </si>
+  <si>
     <t xml:space="preserve">BEYOND TOMORROW ASSUMPTIONS</t>
   </si>
   <si>
@@ -271,6 +284,180 @@
   </si>
   <si>
     <t xml:space="preserve">Remaining to raise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIVE SHOW SPONSORSHIP (weekly YouTube show)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edit the yellow cells. Bottom-up build of the live show sponsor tiers (Noa, 18 Oct 2026). Pick a scenario in B4. B5 decides whether the show sits inside the existing sponsor lines on Assumptions (default, deck totals unchanged) or is added on top.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario (1 Floor, 2 Base, 3 Ceiling)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Floor = 1x $6k + 1x $8k, the minimum Noa expects to sign. Base ramps to 1 of each tier. Ceiling = every slot sold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Treatment (1 inside existing sponsor lines, 2 on top)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 keeps total revenue as in the deck and shows how much of it the show backs. 2 adds the show to revenue; only right if these sponsors are not already in rows 10 to 12 of Assumptions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Episodes per month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly show, 4 a month initially (sponsor slide)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Views per episode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target on the sponsor slide (+30k streams per episode). Not yet a track record; sponsors will ask to see it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price uplift per year from 2028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prices held flat. Growth past the ceiling needs price rises backed by views, since slots are capped</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Months sponsored in 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show not launched as of 19 Oct 2026. Set to 1 or 2 if a sponsor signs for Nov or Dec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIER PRICES (USD per month, per sponsor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max per show</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Presented By' read, logo, clips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exclusive by nature: 1 per show</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rolling footer banner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumed max 2 before the screen gets crowded; confirm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intermittent footer banner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumed max 2; confirm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPONSORS PER TIER (average over the year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario / tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Floor: Presented By</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noa minimum: 1x $8k and 1x $6k, held flat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Floor: Rolling footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Floor: Intermittent footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base: Presented By</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Floor at launch, Presented By from mid 2027, a second banner of each kind by 2029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base: Rolling footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base: Intermittent footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceiling: Presented By</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every slot sold: 1 Presented By, 2 of each banner ($38k a month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceiling: Rolling footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceiling: Intermittent footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SELECTED SCENARIO (calculated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sponsors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presented By</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rolling footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intermittent footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REVENUE (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average per month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied price per 1,000 views, all sponsors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sponsor tiers combined. Host read YouTube placements are commonly quoted at roughly $20 to $50 per 1,000 views (approximate, not sourced). A figure far above that needs proof of a premium audience</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOW THE SHOW SITS IN THE MODEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sponsorship in the model (flagship 1 + 2 + mid tier)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">of which live show, bottom up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">of which still to be won</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of sponsorship backed by the live show</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHECKS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presented By sold within the cap per show</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banners sold within the cap per show</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inside mode: show fits inside the existing sponsor lines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario and treatment are valid choices</t>
   </si>
   <si>
     <t xml:space="preserve">CONSOLIDATED P&amp;L (calculated)</t>
@@ -316,13 +503,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
-    <numFmt numFmtId="166" formatCode="0%"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="\$#,##0"/>
+    <numFmt numFmtId="167" formatCode="0%"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="0"/>
+    <numFmt numFmtId="170" formatCode="#,##0"/>
+    <numFmt numFmtId="171" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -403,6 +594,13 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
       <color rgb="FF0A1730"/>
       <name val="Cambria"/>
       <family val="0"/>
@@ -475,7 +673,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -520,7 +718,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -532,15 +734,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -552,15 +750,43 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -568,15 +794,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -832,7 +1058,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultColWidth="8.515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
@@ -1083,9 +1309,104 @@
         <v>PASS</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>2028</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>2029</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="str">
+        <f aca="false">"Live show ("&amp;CHOOSE('Live show'!$B$4,"floor","base","ceiling")&amp;" case)"</f>
+        <v>Live show (base case)</v>
+      </c>
+      <c r="B27" s="11" t="n">
+        <f aca="false">'Live show'!B40</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="11" t="n">
+        <f aca="false">'Live show'!C40</f>
+        <v>228000</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <f aca="false">'Live show'!D40</f>
+        <v>384000</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <f aca="false">'Live show'!E40</f>
+        <v>456000</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" s="11" t="n">
+        <f aca="false">'Live show'!B48</f>
+        <v>240000</v>
+      </c>
+      <c r="C28" s="11" t="n">
+        <f aca="false">'Live show'!C48</f>
+        <v>1102000</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <f aca="false">'Live show'!D48</f>
+        <v>2620000</v>
+      </c>
+      <c r="E28" s="11" t="n">
+        <f aca="false">'Live show'!E48</f>
+        <v>8544000</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="12" t="n">
+        <f aca="false">'Live show'!B49</f>
+        <v>0</v>
+      </c>
+      <c r="C29" s="12" t="n">
+        <f aca="false">'Live show'!C49</f>
+        <v>0.171428571428571</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <f aca="false">'Live show'!D49</f>
+        <v>0.127829560585886</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <f aca="false">'Live show'!E49</f>
+        <v>0.0506666666666667</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B30" s="1" t="str">
+        <f aca="false">IF(COUNTIF('Live show'!B53:E56,"FAIL")=0,"PASS","FAIL")</f>
+        <v>PASS</v>
       </c>
     </row>
   </sheetData>
@@ -1113,78 +1434,78 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>18</v>
+      <c r="A1" s="13" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="B3" s="14" t="n">
         <v>1500000</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="13" t="n">
+        <v>26</v>
+      </c>
+      <c r="B4" s="14" t="n">
         <v>11000000</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="13" t="n">
+        <v>27</v>
+      </c>
+      <c r="B5" s="14" t="n">
         <v>660000</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="14" t="n">
+        <v>29</v>
+      </c>
+      <c r="B6" s="15" t="n">
         <v>0.2</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="15" t="n">
+        <v>31</v>
+      </c>
+      <c r="B7" s="16" t="n">
         <v>0.008</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>2026</v>
@@ -1199,217 +1520,217 @@
         <v>2029</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="13" t="n">
+        <v>36</v>
+      </c>
+      <c r="B10" s="14" t="n">
         <v>100000</v>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="14" t="n">
         <v>520000</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>1304000</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="14" t="n">
         <v>4000000</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B11" s="13" t="n">
+        <v>38</v>
+      </c>
+      <c r="B11" s="14" t="n">
         <v>80000</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="14" t="n">
         <v>460000</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>1000000</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="14" t="n">
         <v>3200000</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="13" t="n">
+        <v>39</v>
+      </c>
+      <c r="B12" s="14" t="n">
         <v>60000</v>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="14" t="n">
         <v>350000</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <v>700000</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="14" t="n">
         <v>1800000</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="B13" s="14" t="n">
         <v>40000</v>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="14" t="n">
         <v>250000</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="14" t="n">
         <v>500000</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="14" t="n">
         <v>1500000</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="13" t="n">
+        <v>42</v>
+      </c>
+      <c r="B14" s="14" t="n">
         <v>20000</v>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C14" s="14" t="n">
         <v>220000</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="14" t="n">
         <v>400000</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="14" t="n">
         <v>1080000</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" s="13" t="n">
+        <v>44</v>
+      </c>
+      <c r="B15" s="14" t="n">
         <v>130000</v>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="14" t="n">
         <v>500000</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="14" t="n">
         <v>700000</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="14" t="n">
         <v>1000000</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="13" t="n">
+        <v>46</v>
+      </c>
+      <c r="B16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="14" t="n">
         <v>1100000</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="14" t="n">
         <v>2300000</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="14" t="n">
         <v>7000000</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B17" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="13" t="n">
+        <v>48</v>
+      </c>
+      <c r="B17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="14" t="n">
         <v>1000000</v>
       </c>
-      <c r="E17" s="13" t="n">
+      <c r="E17" s="14" t="n">
         <v>2700000</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B18" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="14" t="n">
         <v>12000000</v>
       </c>
-      <c r="E18" s="13" t="n">
+      <c r="E18" s="14" t="n">
         <v>40000000</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B19" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="13" t="n">
+        <v>52</v>
+      </c>
+      <c r="B19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B22" s="5" t="n">
         <v>2026</v>
@@ -1424,251 +1745,251 @@
         <v>2029</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B23" s="13" t="n">
+        <v>55</v>
+      </c>
+      <c r="B23" s="14" t="n">
         <v>280000</v>
       </c>
-      <c r="C23" s="13" t="n">
+      <c r="C23" s="14" t="n">
         <v>1300000</v>
       </c>
-      <c r="D23" s="13" t="n">
+      <c r="D23" s="14" t="n">
         <v>2000000</v>
       </c>
-      <c r="E23" s="13" t="n">
+      <c r="E23" s="14" t="n">
         <v>4000000</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" s="13" t="n">
+        <v>57</v>
+      </c>
+      <c r="B24" s="14" t="n">
         <v>80000</v>
       </c>
-      <c r="C24" s="13" t="n">
+      <c r="C24" s="14" t="n">
         <v>750000</v>
       </c>
-      <c r="D24" s="13" t="n">
+      <c r="D24" s="14" t="n">
         <v>1500000</v>
       </c>
-      <c r="E24" s="13" t="n">
+      <c r="E24" s="14" t="n">
         <v>3800000</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B25" s="13" t="n">
+        <v>59</v>
+      </c>
+      <c r="B25" s="14" t="n">
         <v>130000</v>
       </c>
-      <c r="C25" s="13" t="n">
+      <c r="C25" s="14" t="n">
         <v>850000</v>
       </c>
-      <c r="D25" s="13" t="n">
+      <c r="D25" s="14" t="n">
         <v>1600000</v>
       </c>
-      <c r="E25" s="13" t="n">
+      <c r="E25" s="14" t="n">
         <v>2400000</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="13" t="n">
+        <v>61</v>
+      </c>
+      <c r="B26" s="14" t="n">
         <v>40000</v>
       </c>
-      <c r="C26" s="13" t="n">
+      <c r="C26" s="14" t="n">
         <v>350000</v>
       </c>
-      <c r="D26" s="13" t="n">
+      <c r="D26" s="14" t="n">
         <v>400000</v>
       </c>
-      <c r="E26" s="13" t="n">
+      <c r="E26" s="14" t="n">
         <v>900000</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="13" t="n">
+        <v>63</v>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="14" t="n">
         <v>500000</v>
       </c>
-      <c r="E27" s="13" t="n">
+      <c r="E27" s="14" t="n">
         <v>1350000</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B28" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="13" t="n">
+        <v>65</v>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="14" t="n">
         <v>60000</v>
       </c>
-      <c r="D28" s="13" t="n">
+      <c r="D28" s="14" t="n">
         <v>120000</v>
       </c>
-      <c r="E28" s="13" t="n">
+      <c r="E28" s="14" t="n">
         <v>200000</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B29" s="13" t="n">
+        <v>67</v>
+      </c>
+      <c r="B29" s="14" t="n">
         <v>30000</v>
       </c>
-      <c r="C29" s="13" t="n">
+      <c r="C29" s="14" t="n">
         <v>90000</v>
       </c>
-      <c r="D29" s="13" t="n">
+      <c r="D29" s="14" t="n">
         <v>250000</v>
       </c>
-      <c r="E29" s="13" t="n">
+      <c r="E29" s="14" t="n">
         <v>500000</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B30" s="13" t="n">
+        <v>68</v>
+      </c>
+      <c r="B30" s="14" t="n">
         <v>30000</v>
       </c>
-      <c r="C30" s="13" t="n">
+      <c r="C30" s="14" t="n">
         <v>60000</v>
       </c>
-      <c r="D30" s="13" t="n">
+      <c r="D30" s="14" t="n">
         <v>120000</v>
       </c>
-      <c r="E30" s="13" t="n">
+      <c r="E30" s="14" t="n">
         <v>250000</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B34" s="13" t="n">
+        <v>73</v>
+      </c>
+      <c r="B34" s="14" t="n">
         <v>600000</v>
       </c>
-      <c r="C34" s="16" t="n">
+      <c r="C34" s="12" t="n">
         <f aca="false">B34/$B$3</f>
         <v>0.4</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B35" s="13" t="n">
+        <v>75</v>
+      </c>
+      <c r="B35" s="14" t="n">
         <v>525000</v>
       </c>
-      <c r="C35" s="16" t="n">
+      <c r="C35" s="12" t="n">
         <f aca="false">B35/$B$3</f>
         <v>0.35</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B36" s="13" t="n">
+        <v>77</v>
+      </c>
+      <c r="B36" s="14" t="n">
         <v>225000</v>
       </c>
-      <c r="C36" s="16" t="n">
+      <c r="C36" s="12" t="n">
         <f aca="false">B36/$B$3</f>
         <v>0.15</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B37" s="13" t="n">
+        <v>79</v>
+      </c>
+      <c r="B37" s="14" t="n">
         <v>150000</v>
       </c>
-      <c r="C37" s="16" t="n">
+      <c r="C37" s="12" t="n">
         <f aca="false">B37/$B$3</f>
         <v>0.1</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="17" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B38" s="18" t="n">
         <f aca="false">SUM(B34:B37)</f>
@@ -1681,7 +2002,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B39" s="1" t="str">
         <f aca="false">IF(ABS(B38-$B$3)&lt;1,"PASS","FAIL")</f>
@@ -1690,23 +2011,23 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B42" s="13" t="n">
+        <v>84</v>
+      </c>
+      <c r="B42" s="14" t="n">
         <v>20000</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B43" s="7" t="n">
         <f aca="false">B3-B5</f>
@@ -1727,6 +2048,802 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F56"/>
+  <sheetFormatPr defaultColWidth="8.515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="78"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B13" s="22" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="22" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C14" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" s="22" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>2028</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>2029</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B22" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D22" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B23" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B24" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B26" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B27" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>2028</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>2029</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B31" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,B19,B22,B25)</f>
+        <v>0</v>
+      </c>
+      <c r="C31" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,C19,C22,C25)</f>
+        <v>0.5</v>
+      </c>
+      <c r="D31" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,D19,D22,D25)</f>
+        <v>1</v>
+      </c>
+      <c r="E31" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,E19,E22,E25)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B32" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,B20,B23,B26)</f>
+        <v>1</v>
+      </c>
+      <c r="C32" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,C20,C23,C26)</f>
+        <v>1</v>
+      </c>
+      <c r="D32" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,D20,D23,D26)</f>
+        <v>2</v>
+      </c>
+      <c r="E32" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,E20,E23,E26)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B33" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,B21,B24,B27)</f>
+        <v>1</v>
+      </c>
+      <c r="C33" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,C21,C24,C27)</f>
+        <v>1</v>
+      </c>
+      <c r="D33" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,D21,D24,D27)</f>
+        <v>1</v>
+      </c>
+      <c r="E33" s="24" t="n">
+        <f aca="false">CHOOSE($B$4,E21,E24,E27)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>2028</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>2029</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B37" s="11" t="n">
+        <f aca="false">B31*$B$13*$B$9*(1+$B$8)^MAX(0,B$36-2027)</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="11" t="n">
+        <f aca="false">C31*$B$13*12*(1+$B$8)^MAX(0,C$36-2027)</f>
+        <v>60000</v>
+      </c>
+      <c r="D37" s="11" t="n">
+        <f aca="false">D31*$B$13*12*(1+$B$8)^MAX(0,D$36-2027)</f>
+        <v>120000</v>
+      </c>
+      <c r="E37" s="11" t="n">
+        <f aca="false">E31*$B$13*12*(1+$B$8)^MAX(0,E$36-2027)</f>
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B38" s="11" t="n">
+        <f aca="false">B32*$B$14*$B$9*(1+$B$8)^MAX(0,B$36-2027)</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="11" t="n">
+        <f aca="false">C32*$B$14*12*(1+$B$8)^MAX(0,C$36-2027)</f>
+        <v>96000</v>
+      </c>
+      <c r="D38" s="11" t="n">
+        <f aca="false">D32*$B$14*12*(1+$B$8)^MAX(0,D$36-2027)</f>
+        <v>192000</v>
+      </c>
+      <c r="E38" s="11" t="n">
+        <f aca="false">E32*$B$14*12*(1+$B$8)^MAX(0,E$36-2027)</f>
+        <v>192000</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B39" s="11" t="n">
+        <f aca="false">B33*$B$15*$B$9*(1+$B$8)^MAX(0,B$36-2027)</f>
+        <v>0</v>
+      </c>
+      <c r="C39" s="11" t="n">
+        <f aca="false">C33*$B$15*12*(1+$B$8)^MAX(0,C$36-2027)</f>
+        <v>72000</v>
+      </c>
+      <c r="D39" s="11" t="n">
+        <f aca="false">D33*$B$15*12*(1+$B$8)^MAX(0,D$36-2027)</f>
+        <v>72000</v>
+      </c>
+      <c r="E39" s="11" t="n">
+        <f aca="false">E33*$B$15*12*(1+$B$8)^MAX(0,E$36-2027)</f>
+        <v>144000</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="26" t="n">
+        <f aca="false">SUM(B37:B39)</f>
+        <v>0</v>
+      </c>
+      <c r="C40" s="26" t="n">
+        <f aca="false">SUM(C37:C39)</f>
+        <v>228000</v>
+      </c>
+      <c r="D40" s="26" t="n">
+        <f aca="false">SUM(D37:D39)</f>
+        <v>384000</v>
+      </c>
+      <c r="E40" s="26" t="n">
+        <f aca="false">SUM(E37:E39)</f>
+        <v>456000</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B41" s="11" t="n">
+        <f aca="false">IFERROR(B40/$B$9,0)</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="11" t="n">
+        <f aca="false">IFERROR(C40/12,0)</f>
+        <v>19000</v>
+      </c>
+      <c r="D41" s="11" t="n">
+        <f aca="false">IFERROR(D40/12,0)</f>
+        <v>32000</v>
+      </c>
+      <c r="E41" s="11" t="n">
+        <f aca="false">IFERROR(E40/12,0)</f>
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B42" s="11" t="n">
+        <f aca="false">IFERROR(B41/($B$6*$B$7/1000),0)</f>
+        <v>0</v>
+      </c>
+      <c r="C42" s="11" t="n">
+        <f aca="false">IFERROR(C41/($B$6*$B$7/1000),0)</f>
+        <v>158.333333333333</v>
+      </c>
+      <c r="D42" s="11" t="n">
+        <f aca="false">IFERROR(D41/($B$6*$B$7/1000),0)</f>
+        <v>266.666666666667</v>
+      </c>
+      <c r="E42" s="11" t="n">
+        <f aca="false">IFERROR(E41/($B$6*$B$7/1000),0)</f>
+        <v>316.666666666667</v>
+      </c>
+      <c r="F42" s="10" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="8" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B45" s="4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>2028</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>2029</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B46" s="11" t="n">
+        <f aca="false">SUM(Assumptions!B10:B12)+IF($B$5=2,B40,0)</f>
+        <v>240000</v>
+      </c>
+      <c r="C46" s="11" t="n">
+        <f aca="false">SUM(Assumptions!C10:C12)+IF($B$5=2,C40,0)</f>
+        <v>1330000</v>
+      </c>
+      <c r="D46" s="11" t="n">
+        <f aca="false">SUM(Assumptions!D10:D12)+IF($B$5=2,D40,0)</f>
+        <v>3004000</v>
+      </c>
+      <c r="E46" s="11" t="n">
+        <f aca="false">SUM(Assumptions!E10:E12)+IF($B$5=2,E40,0)</f>
+        <v>9000000</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B47" s="11" t="n">
+        <f aca="false">B40</f>
+        <v>0</v>
+      </c>
+      <c r="C47" s="11" t="n">
+        <f aca="false">C40</f>
+        <v>228000</v>
+      </c>
+      <c r="D47" s="11" t="n">
+        <f aca="false">D40</f>
+        <v>384000</v>
+      </c>
+      <c r="E47" s="11" t="n">
+        <f aca="false">E40</f>
+        <v>456000</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B48" s="11" t="n">
+        <f aca="false">B46-B47</f>
+        <v>240000</v>
+      </c>
+      <c r="C48" s="11" t="n">
+        <f aca="false">C46-C47</f>
+        <v>1102000</v>
+      </c>
+      <c r="D48" s="11" t="n">
+        <f aca="false">D46-D47</f>
+        <v>2620000</v>
+      </c>
+      <c r="E48" s="11" t="n">
+        <f aca="false">E46-E47</f>
+        <v>8544000</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B49" s="12" t="n">
+        <f aca="false">IFERROR(B47/B46,0)</f>
+        <v>0</v>
+      </c>
+      <c r="C49" s="12" t="n">
+        <f aca="false">IFERROR(C47/C46,0)</f>
+        <v>0.171428571428571</v>
+      </c>
+      <c r="D49" s="12" t="n">
+        <f aca="false">IFERROR(D47/D46,0)</f>
+        <v>0.127829560585886</v>
+      </c>
+      <c r="E49" s="12" t="n">
+        <f aca="false">IFERROR(E47/E46,0)</f>
+        <v>0.0506666666666667</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B52" s="4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D52" s="4" t="n">
+        <v>2028</v>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>2029</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B53" s="1" t="str">
+        <f aca="false">IF(B31&lt;=$C$13,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="C53" s="1" t="str">
+        <f aca="false">IF(C31&lt;=$C$13,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="D53" s="1" t="str">
+        <f aca="false">IF(D31&lt;=$C$13,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="E53" s="1" t="str">
+        <f aca="false">IF(E31&lt;=$C$13,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B54" s="1" t="str">
+        <f aca="false">IF(AND(B32&lt;=$C$14,B33&lt;=$C$15),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="C54" s="1" t="str">
+        <f aca="false">IF(AND(C32&lt;=$C$14,C33&lt;=$C$15),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="D54" s="1" t="str">
+        <f aca="false">IF(AND(D32&lt;=$C$14,D33&lt;=$C$15),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="E54" s="1" t="str">
+        <f aca="false">IF(AND(E32&lt;=$C$14,E33&lt;=$C$15),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B55" s="1" t="str">
+        <f aca="false">IF(OR($B$5=2,B40&lt;=SUM(Assumptions!B10:B12)),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="C55" s="1" t="str">
+        <f aca="false">IF(OR($B$5=2,C40&lt;=SUM(Assumptions!C10:C12)),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="D55" s="1" t="str">
+        <f aca="false">IF(OR($B$5=2,D40&lt;=SUM(Assumptions!D10:D12)),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="E55" s="1" t="str">
+        <f aca="false">IF(OR($B$5=2,E40&lt;=SUM(Assumptions!E10:E12)),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B56" s="1" t="str">
+        <f aca="false">IF(AND(OR($B$4=1,$B$4=2,$B$4=3),OR($B$5=1,$B$5=2)),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="C56" s="1" t="str">
+        <f aca="false">IF(AND(OR($B$4=1,$B$4=2,$B$4=3),OR($B$5=1,$B$5=2)),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="D56" s="1" t="str">
+        <f aca="false">IF(AND(OR($B$4=1,$B$4=2,$B$4=3),OR($B$5=1,$B$5=2)),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="E56" s="1" t="str">
+        <f aca="false">IF(AND(OR($B$4=1,$B$4=2,$B$4=3),OR($B$5=1,$B$5=2)),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E28"/>
@@ -1737,8 +2854,8 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>83</v>
+      <c r="A1" s="13" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1763,25 +2880,25 @@
         <v>4</v>
       </c>
       <c r="B4" s="7" t="n">
-        <f aca="false">SUM(Assumptions!B10:B14)</f>
+        <f aca="false">SUM(Assumptions!B10:B14)+IF('Live show'!$B$5=2,'Live show'!B40,0)</f>
         <v>300000</v>
       </c>
       <c r="C4" s="7" t="n">
-        <f aca="false">SUM(Assumptions!C10:C14)</f>
+        <f aca="false">SUM(Assumptions!C10:C14)+IF('Live show'!$B$5=2,'Live show'!C40,0)</f>
         <v>1800000</v>
       </c>
       <c r="D4" s="7" t="n">
-        <f aca="false">SUM(Assumptions!D10:D14)</f>
+        <f aca="false">SUM(Assumptions!D10:D14)+IF('Live show'!$B$5=2,'Live show'!D40,0)</f>
         <v>3904000</v>
       </c>
       <c r="E4" s="7" t="n">
-        <f aca="false">SUM(Assumptions!E10:E14)</f>
+        <f aca="false">SUM(Assumptions!E10:E14)+IF('Live show'!$B$5=2,'Live show'!E40,0)</f>
         <v>11580000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="B5" s="7" t="n">
         <f aca="false">SUM(Assumptions!B15:B16)</f>
@@ -1802,7 +2919,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">Assumptions!B17</f>
@@ -1822,22 +2939,22 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="B7" s="21" t="n">
+      <c r="A7" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="B7" s="28" t="n">
         <f aca="false">B4+B5+B6</f>
         <v>430000</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="28" t="n">
         <f aca="false">C4+C5+C6</f>
         <v>3400000</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="28" t="n">
         <f aca="false">D4+D5+D6</f>
         <v>7904000</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="28" t="n">
         <f aca="false">E4+E5+E6</f>
         <v>22280000</v>
       </c>
@@ -1866,7 +2983,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="B9" s="7" t="n">
         <f aca="false">Assumptions!B19</f>
@@ -1886,22 +3003,22 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
-        <v>88</v>
-      </c>
-      <c r="B10" s="21" t="n">
+      <c r="A10" s="27" t="s">
+        <v>150</v>
+      </c>
+      <c r="B10" s="28" t="n">
         <f aca="false">B8+B9</f>
         <v>0</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="28" t="n">
         <f aca="false">C8+C9</f>
         <v>0</v>
       </c>
-      <c r="D10" s="21" t="n">
+      <c r="D10" s="28" t="n">
         <f aca="false">D8+D9</f>
         <v>96000</v>
       </c>
-      <c r="E10" s="21" t="n">
+      <c r="E10" s="28" t="n">
         <f aca="false">E8+E9</f>
         <v>320000</v>
       </c>
@@ -1910,26 +3027,26 @@
       <c r="A11" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="29" t="n">
         <f aca="false">B7+B10</f>
         <v>430000</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="29" t="n">
         <f aca="false">C7+C10</f>
         <v>3400000</v>
       </c>
-      <c r="D11" s="22" t="n">
+      <c r="D11" s="29" t="n">
         <f aca="false">D7+D10</f>
         <v>8000000</v>
       </c>
-      <c r="E11" s="22" t="n">
+      <c r="E11" s="29" t="n">
         <f aca="false">E7+E10</f>
         <v>22600000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B12" s="7" t="n">
         <f aca="false">Assumptions!B23</f>
@@ -1950,7 +3067,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B13" s="7" t="n">
         <f aca="false">Assumptions!B24</f>
@@ -1971,7 +3088,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B14" s="7" t="n">
         <f aca="false">Assumptions!B25</f>
@@ -1992,7 +3109,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B15" s="7" t="n">
         <f aca="false">Assumptions!B26</f>
@@ -2013,7 +3130,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B16" s="7" t="n">
         <f aca="false">Assumptions!B27</f>
@@ -2034,7 +3151,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B17" s="7" t="n">
         <f aca="false">Assumptions!B28</f>
@@ -2055,7 +3172,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">Assumptions!B29</f>
@@ -2076,7 +3193,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B19" s="7" t="n">
         <f aca="false">Assumptions!B30</f>
@@ -2096,71 +3213,71 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="B20" s="21" t="n">
+      <c r="A20" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="B20" s="28" t="n">
         <f aca="false">SUM(B12:B19)</f>
         <v>590000</v>
       </c>
-      <c r="C20" s="21" t="n">
+      <c r="C20" s="28" t="n">
         <f aca="false">SUM(C12:C19)</f>
         <v>3460000</v>
       </c>
-      <c r="D20" s="21" t="n">
+      <c r="D20" s="28" t="n">
         <f aca="false">SUM(D12:D19)</f>
         <v>6490000</v>
       </c>
-      <c r="E20" s="21" t="n">
+      <c r="E20" s="28" t="n">
         <f aca="false">SUM(E12:E19)</f>
         <v>13400000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="21" t="n">
+      <c r="B21" s="28" t="n">
         <f aca="false">B11-B20</f>
         <v>-160000</v>
       </c>
-      <c r="C21" s="21" t="n">
+      <c r="C21" s="28" t="n">
         <f aca="false">C11-C20</f>
         <v>-60000</v>
       </c>
-      <c r="D21" s="21" t="n">
+      <c r="D21" s="28" t="n">
         <f aca="false">D11-D20</f>
         <v>1510000</v>
       </c>
-      <c r="E21" s="21" t="n">
+      <c r="E21" s="28" t="n">
         <f aca="false">E11-E20</f>
         <v>9200000</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B22" s="23" t="n">
+        <v>152</v>
+      </c>
+      <c r="B22" s="30" t="n">
         <f aca="false">IFERROR(B21/B11,0)</f>
         <v>-0.372093023255814</v>
       </c>
-      <c r="C22" s="23" t="n">
+      <c r="C22" s="30" t="n">
         <f aca="false">IFERROR(C21/C11,0)</f>
         <v>-0.0176470588235294</v>
       </c>
-      <c r="D22" s="23" t="n">
+      <c r="D22" s="30" t="n">
         <f aca="false">IFERROR(D21/D11,0)</f>
         <v>0.18875</v>
       </c>
-      <c r="E22" s="23" t="n">
+      <c r="E22" s="30" t="n">
         <f aca="false">IFERROR(E21/E11,0)</f>
         <v>0.407079646017699</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>91</v>
+        <v>153</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">-MAX(0,B21)*Assumptions!$B$6</f>
@@ -2180,29 +3297,29 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="24" t="s">
-        <v>92</v>
-      </c>
-      <c r="B24" s="25" t="n">
+      <c r="A24" s="31" t="s">
+        <v>154</v>
+      </c>
+      <c r="B24" s="32" t="n">
         <f aca="false">B21+B23</f>
         <v>-160000</v>
       </c>
-      <c r="C24" s="25" t="n">
+      <c r="C24" s="32" t="n">
         <f aca="false">C21+C23</f>
         <v>-60000</v>
       </c>
-      <c r="D24" s="25" t="n">
+      <c r="D24" s="32" t="n">
         <f aca="false">D21+D23</f>
         <v>1208000</v>
       </c>
-      <c r="E24" s="25" t="n">
+      <c r="E24" s="32" t="n">
         <f aca="false">E21+E23</f>
         <v>7360000</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>93</v>
+        <v>155</v>
       </c>
       <c r="B25" s="7" t="n">
         <v>0</v>
@@ -2222,7 +3339,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>94</v>
+        <v>156</v>
       </c>
       <c r="B26" s="7" t="n">
         <f aca="false">Assumptions!$B$3</f>
@@ -2240,7 +3357,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>95</v>
+        <v>157</v>
       </c>
       <c r="B27" s="7" t="n">
         <f aca="false">B24</f>
@@ -2260,22 +3377,22 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="21" t="n">
+      <c r="B28" s="28" t="n">
         <f aca="false">B25+B26+B27</f>
         <v>1340000</v>
       </c>
-      <c r="C28" s="21" t="n">
+      <c r="C28" s="28" t="n">
         <f aca="false">C25+C26+C27</f>
         <v>1280000</v>
       </c>
-      <c r="D28" s="21" t="n">
+      <c r="D28" s="28" t="n">
         <f aca="false">D25+D26+D27</f>
         <v>2488000</v>
       </c>
-      <c r="E28" s="21" t="n">
+      <c r="E28" s="28" t="n">
         <f aca="false">E25+E26+E27</f>
         <v>9848000</v>
       </c>

</xml_diff>